<commit_message>
Added agents in the project
</commit_message>
<xml_diff>
--- a/testdata/testdata1.xlsx
+++ b/testdata/testdata1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="6900"/>
+    <workbookView windowWidth="20490" windowHeight="7020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="27">
   <si>
     <t>TestCase</t>
   </si>
@@ -62,10 +62,10 @@
     <t>D2C_Ticket</t>
   </si>
   <si>
-    <t>https://rims-demo.blubirch.com</t>
-  </si>
-  <si>
-    <t>CSE02</t>
+    <t>https://qa-crompton-rims-k8s.blubirch.com/</t>
+  </si>
+  <si>
+    <t>dava_admin</t>
   </si>
   <si>
     <t>blubirch@123</t>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>Reverse logistics</t>
-  </si>
-  <si>
-    <t>dava_admin</t>
   </si>
   <si>
     <t>PRD</t>
@@ -760,7 +757,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1123,7 +1120,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="2">
-        <v>493666367</v>
+        <v>89234794</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>14</v>
@@ -1167,7 +1164,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1181,7 +1178,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1192,7 +1189,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1200,18 +1197,18 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>13</v>
@@ -1220,9 +1217,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" display="https://qa-fta.web.app/login" tooltip="https://qa-fta.web.app/login"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://rims-demo.blubirch.com"/>
-    <hyperlink ref="B4" r:id="rId2" display="https://rims-demo.blubirch.com"/>
-    <hyperlink ref="B6" r:id="rId2" display="https://rims-demo.blubirch.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>